<commit_message>
Yeni arıza bildir sayfasından 'FRACAS sistemine yeni arıza kaydı ekleyin' yazısını sil
</commit_message>
<xml_diff>
--- a/data/belgrad/Veriler.xlsx
+++ b/data/belgrad/Veriler.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\belgrad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2541FF59-46A0-4433-AD50-8AFFE15E4E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{186DB1E5-615C-4317-9BF4-AE0E5BBEC9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2784" yWindow="3456" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -2399,6 +2399,7 @@
     <col min="4" max="4" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.33203125" customWidth="1"/>
     <col min="6" max="6" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Debug: API'ye ultra detaylı loglar ekle - sütun adlar, normalize, eşleşme, filtre sonrası detay
</commit_message>
<xml_diff>
--- a/data/belgrad/Veriler.xlsx
+++ b/data/belgrad/Veriler.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Downloads\bozankaya_ssh_takip (1)\bozankaya_ssh_takip\data\belgrad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\belgrad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BAA79B-C0CA-4500-901D-9D2371C8C714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61F2F6D-DB29-42AF-A000-DDEE0BD6DA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,25 @@
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
     <sheet name="Sayfa2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="200">
   <si>
     <t>Traction_Converter</t>
   </si>
@@ -584,6 +597,9 @@
     <t>(I) İlk Defa Karşılaşılan Arıza</t>
   </si>
   <si>
+    <t>BELGRAD</t>
+  </si>
+  <si>
     <t>SA</t>
   </si>
   <si>
@@ -617,15 +633,16 @@
     <t>M</t>
   </si>
   <si>
-    <t>BELGRAD</t>
+    <t>İşçilik</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-41F]d\ mmmm\ yy;@"/>
+    <numFmt numFmtId="165" formatCode="_-[$£-809]* #,##0.00_-;\-[$£-809]* #,##0.00_-;_-[$£-809]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -784,7 +801,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -833,6 +850,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2315,15 +2333,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.33203125" customWidth="1"/>
     <col min="5" max="5" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>177</v>
       </c>
@@ -2342,8 +2361,11 @@
       <c r="F1" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1531</v>
       </c>
@@ -2362,109 +2384,112 @@
       <c r="F2" s="17" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="18">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1532</v>
       </c>
       <c r="B3" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1533</v>
       </c>
       <c r="C4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>1534</v>
       </c>
       <c r="C5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D5" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>1535</v>
       </c>
       <c r="C6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1536</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1537</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>1538</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1539</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>1540</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>1541</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>1542</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1543</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>1544</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>1545</v>
       </c>

</xml_diff>

<commit_message>
v4.1: MTTR hesaplama tamamlandı - tüm projeler için tamir süresi Excel'den çekiliyor, optimize edilmeden önceki güvenli checkpoint
</commit_message>
<xml_diff>
--- a/data/belgrad/Veriler.xlsx
+++ b/data/belgrad/Veriler.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\belgrad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61F2F6D-DB29-42AF-A000-DDEE0BD6DA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96940289-A0E0-4E0D-9A51-5541C628CA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="201">
   <si>
     <t>Traction_Converter</t>
   </si>
@@ -634,6 +634,9 @@
   </si>
   <si>
     <t>İşçilik</t>
+  </si>
+  <si>
+    <t>Buzzer</t>
   </si>
 </sst>
 </file>
@@ -1513,6 +1516,9 @@
       <c r="AL3" s="11"/>
       <c r="AM3" s="10"/>
       <c r="AN3" s="10"/>
+      <c r="AO3" s="10" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="4" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
@@ -1591,6 +1597,7 @@
       <c r="AL4" s="11"/>
       <c r="AM4" s="10"/>
       <c r="AN4" s="10"/>
+      <c r="AO4" s="10"/>
     </row>
     <row r="5" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
@@ -1663,6 +1670,7 @@
       <c r="AL5" s="11"/>
       <c r="AM5" s="10"/>
       <c r="AN5" s="10"/>
+      <c r="AO5" s="10"/>
     </row>
     <row r="6" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
@@ -1733,6 +1741,7 @@
       <c r="AL6" s="11"/>
       <c r="AM6" s="10"/>
       <c r="AN6" s="10"/>
+      <c r="AO6" s="10"/>
     </row>
     <row r="7" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
@@ -1799,6 +1808,7 @@
       <c r="AL7" s="11"/>
       <c r="AM7" s="10"/>
       <c r="AN7" s="10"/>
+      <c r="AO7" s="10"/>
     </row>
     <row r="8" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
@@ -1859,6 +1869,7 @@
       <c r="AL8" s="11"/>
       <c r="AM8" s="10"/>
       <c r="AN8" s="10"/>
+      <c r="AO8" s="10"/>
     </row>
     <row r="9" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
@@ -1917,6 +1928,7 @@
       <c r="AL9" s="11"/>
       <c r="AM9" s="10"/>
       <c r="AN9" s="10"/>
+      <c r="AO9" s="10"/>
     </row>
     <row r="10" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
@@ -1971,6 +1983,7 @@
       <c r="AL10" s="11"/>
       <c r="AM10" s="10"/>
       <c r="AN10" s="10"/>
+      <c r="AO10" s="10"/>
     </row>
     <row r="11" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
@@ -2023,6 +2036,7 @@
       <c r="AL11" s="11"/>
       <c r="AM11" s="10"/>
       <c r="AN11" s="10"/>
+      <c r="AO11" s="10"/>
     </row>
     <row r="12" spans="1:41" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16"/>
@@ -2069,6 +2083,7 @@
       <c r="AL12" s="10"/>
       <c r="AM12" s="10"/>
       <c r="AN12" s="10"/>
+      <c r="AO12" s="10"/>
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>
@@ -2111,6 +2126,7 @@
       <c r="AL13" s="10"/>
       <c r="AM13" s="10"/>
       <c r="AN13" s="10"/>
+      <c r="AO13" s="10"/>
     </row>
     <row r="14" spans="1:41" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
@@ -2155,6 +2171,7 @@
       <c r="AL14" s="10"/>
       <c r="AM14" s="10"/>
       <c r="AN14" s="10"/>
+      <c r="AO14" s="10"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
@@ -2197,6 +2214,7 @@
       <c r="AL15" s="10"/>
       <c r="AM15" s="10"/>
       <c r="AN15" s="10"/>
+      <c r="AO15" s="10"/>
     </row>
     <row r="16" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
@@ -2241,8 +2259,9 @@
       <c r="AL16" s="10"/>
       <c r="AM16" s="10"/>
       <c r="AN16" s="10"/>
-    </row>
-    <row r="17" spans="1:40" x14ac:dyDescent="0.3">
+      <c r="AO16" s="10"/>
+    </row>
+    <row r="17" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
@@ -2283,8 +2302,9 @@
       <c r="AL17" s="10"/>
       <c r="AM17" s="10"/>
       <c r="AN17" s="10"/>
-    </row>
-    <row r="18" spans="1:40" x14ac:dyDescent="0.3">
+      <c r="AO17" s="10"/>
+    </row>
+    <row r="18" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -2325,6 +2345,7 @@
       <c r="AL18" s="10"/>
       <c r="AM18" s="10"/>
       <c r="AN18" s="10"/>
+      <c r="AO18" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>